<commit_message>
Agent compelted with report
</commit_message>
<xml_diff>
--- a/data/SIT Extract -W1-20260625.xlsx
+++ b/data/SIT Extract -W1-20260625.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myoffice.accenture.com/personal/paveen_km_accenture_com/Documents/Desktop/ReportAgentClaude/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9ADD91F3-DB69-4CC1-A618-CE4E94FCEDB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9271D7C3-DD37-48F0-BEF1-9316F69527FB}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{9ADD91F3-DB69-4CC1-A618-CE4E94FCEDB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D34F81E6-B26B-4BA6-A144-E01C3700C362}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Execution-input" sheetId="2" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="145">
   <si>
     <t>Id</t>
   </si>
@@ -459,9 +459,6 @@
   </si>
   <si>
     <t>In Progress</t>
-  </si>
-  <si>
-    <t>Ready for Retest</t>
   </si>
 </sst>
 </file>
@@ -2122,7 +2119,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>130</v>
       </c>
@@ -2142,7 +2139,7 @@
         <v>126</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>124</v>

</xml_diff>